<commit_message>
Add digitized Somoano-Huera-Huarte data
Add CSV datasets digitized from Figures 4–6 for the N=3, cToR=0.32 configuration, update the metadata workbook, and replace the source plot images.
</commit_message>
<xml_diff>
--- a/(Default) Research Papers/!management/metadata.csv.xlsx
+++ b/(Default) Research Papers/!management/metadata.csv.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30527"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Aario\Downloads\Productive files\College\Semester 5\Research\Literature Review\Research Papers\!management\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Aario\Downloads\Productive files\College\Semester 5\Research\vawt-research\(Default) Research Papers\!management\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{61601383-CAF6-4466-BE6A-06E6D2FA547B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D16875BE-D0D8-454B-AC47-5B15BBF4AB73}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{6350385E-C843-4413-9968-6DC09C1E5CFB}"/>
+    <workbookView xWindow="-96" yWindow="0" windowWidth="12252" windowHeight="12336" xr2:uid="{6350385E-C843-4413-9968-6DC09C1E5CFB}"/>
   </bookViews>
   <sheets>
     <sheet name="metadata" sheetId="1" r:id="rId1"/>
@@ -1791,16 +1791,17 @@
     <col min="1" max="1" width="28.44140625" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="54.44140625" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="2.33203125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="9" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="1.33203125" customWidth="1"/>
-    <col min="6" max="6" width="8.5546875" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="1" hidden="1" customWidth="1"/>
-    <col min="8" max="8" width="7.33203125" hidden="1" customWidth="1"/>
-    <col min="9" max="9" width="13.21875" hidden="1" customWidth="1"/>
-    <col min="10" max="10" width="12.88671875" hidden="1" customWidth="1"/>
-    <col min="11" max="11" width="11.6640625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="8.6640625" customWidth="1"/>
+    <col min="5" max="5" width="0.109375" hidden="1" customWidth="1"/>
+    <col min="6" max="6" width="20.44140625" customWidth="1"/>
+    <col min="7" max="7" width="23.33203125" hidden="1" customWidth="1"/>
+    <col min="8" max="8" width="0.109375" hidden="1" customWidth="1"/>
+    <col min="9" max="9" width="30.109375" customWidth="1"/>
+    <col min="10" max="10" width="0.88671875" hidden="1" customWidth="1"/>
+    <col min="11" max="11" width="11.88671875" customWidth="1"/>
     <col min="12" max="12" width="35.77734375" bestFit="1" customWidth="1"/>
     <col min="15" max="15" width="7.44140625" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="37.77734375" bestFit="1" customWidth="1"/>
     <col min="17" max="17" width="64.33203125" bestFit="1" customWidth="1"/>
     <col min="18" max="18" width="16.33203125" bestFit="1" customWidth="1"/>
     <col min="19" max="19" width="17.88671875" bestFit="1" customWidth="1"/>
@@ -5687,1263 +5688,1263 @@
         <v>194</v>
       </c>
     </row>
-    <row r="100" spans="1:21" x14ac:dyDescent="0.3">
-      <c r="A100" t="s">
+    <row r="100" spans="1:21" s="2" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A100" s="2" t="s">
         <v>237</v>
       </c>
-      <c r="B100" t="s">
+      <c r="B100" s="2" t="s">
         <v>238</v>
       </c>
-      <c r="C100">
+      <c r="C100" s="2">
         <v>3</v>
       </c>
-      <c r="D100">
+      <c r="D100" s="2">
         <v>0.32</v>
       </c>
-      <c r="F100">
+      <c r="F100" s="2">
         <v>300000</v>
       </c>
-      <c r="H100">
+      <c r="H100" s="2">
         <v>0</v>
       </c>
-      <c r="L100" t="s">
+      <c r="L100" s="2" t="s">
         <v>184</v>
       </c>
-      <c r="M100" t="s">
+      <c r="M100" s="2" t="s">
         <v>24</v>
       </c>
-      <c r="N100" t="s">
+      <c r="N100" s="2" t="s">
         <v>25</v>
       </c>
-      <c r="O100" t="s">
-        <v>26</v>
-      </c>
-      <c r="P100" t="s">
+      <c r="O100" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="P100" s="2" t="s">
         <v>239</v>
       </c>
-      <c r="Q100" t="s">
+      <c r="Q100" s="2" t="s">
         <v>240</v>
       </c>
-      <c r="T100" t="s">
+      <c r="T100" s="2" t="s">
         <v>101</v>
       </c>
-      <c r="U100" t="s">
+      <c r="U100" s="2" t="s">
         <v>241</v>
       </c>
     </row>
-    <row r="101" spans="1:21" x14ac:dyDescent="0.3">
-      <c r="A101" t="s">
+    <row r="101" spans="1:21" s="2" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A101" s="2" t="s">
         <v>242</v>
       </c>
-      <c r="B101" t="s">
+      <c r="B101" s="2" t="s">
         <v>243</v>
       </c>
-      <c r="C101">
+      <c r="C101" s="2">
         <v>3</v>
       </c>
-      <c r="D101">
+      <c r="D101" s="2">
         <v>0.32</v>
       </c>
-      <c r="F101">
+      <c r="F101" s="2">
         <v>300000</v>
       </c>
-      <c r="H101">
+      <c r="H101" s="2">
         <v>2</v>
       </c>
-      <c r="I101" t="s">
+      <c r="I101" s="2" t="s">
         <v>244</v>
       </c>
-      <c r="L101" t="s">
+      <c r="L101" s="2" t="s">
         <v>184</v>
       </c>
-      <c r="M101" t="s">
+      <c r="M101" s="2" t="s">
         <v>24</v>
       </c>
-      <c r="N101" t="s">
+      <c r="N101" s="2" t="s">
         <v>25</v>
       </c>
-      <c r="O101" t="s">
-        <v>26</v>
-      </c>
-      <c r="P101" t="s">
+      <c r="O101" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="P101" s="2" t="s">
         <v>239</v>
       </c>
-      <c r="Q101" t="s">
+      <c r="Q101" s="2" t="s">
         <v>240</v>
       </c>
-      <c r="T101" t="s">
+      <c r="T101" s="2" t="s">
         <v>101</v>
       </c>
-      <c r="U101" t="s">
+      <c r="U101" s="2" t="s">
         <v>241</v>
       </c>
     </row>
-    <row r="102" spans="1:21" x14ac:dyDescent="0.3">
-      <c r="A102" t="s">
+    <row r="102" spans="1:21" s="2" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A102" s="2" t="s">
         <v>245</v>
       </c>
-      <c r="B102" t="s">
+      <c r="B102" s="2" t="s">
         <v>246</v>
       </c>
-      <c r="C102">
+      <c r="C102" s="2">
         <v>3</v>
       </c>
-      <c r="D102">
+      <c r="D102" s="2">
         <v>0.32</v>
       </c>
-      <c r="F102">
+      <c r="F102" s="2">
         <v>300000</v>
       </c>
-      <c r="H102">
+      <c r="H102" s="2">
         <v>4</v>
       </c>
-      <c r="I102" t="s">
+      <c r="I102" s="2" t="s">
         <v>244</v>
       </c>
-      <c r="L102" t="s">
+      <c r="L102" s="2" t="s">
         <v>184</v>
       </c>
-      <c r="M102" t="s">
+      <c r="M102" s="2" t="s">
         <v>24</v>
       </c>
-      <c r="N102" t="s">
+      <c r="N102" s="2" t="s">
         <v>25</v>
       </c>
-      <c r="O102" t="s">
-        <v>26</v>
-      </c>
-      <c r="P102" t="s">
+      <c r="O102" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="P102" s="2" t="s">
         <v>239</v>
       </c>
-      <c r="Q102" t="s">
+      <c r="Q102" s="2" t="s">
         <v>240</v>
       </c>
-      <c r="T102" t="s">
+      <c r="T102" s="2" t="s">
         <v>101</v>
       </c>
-      <c r="U102" t="s">
+      <c r="U102" s="2" t="s">
         <v>241</v>
       </c>
     </row>
-    <row r="103" spans="1:21" x14ac:dyDescent="0.3">
-      <c r="A103" t="s">
+    <row r="103" spans="1:21" s="2" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A103" s="2" t="s">
         <v>247</v>
       </c>
-      <c r="B103" t="s">
+      <c r="B103" s="2" t="s">
         <v>248</v>
       </c>
-      <c r="C103">
+      <c r="C103" s="2">
         <v>3</v>
       </c>
-      <c r="D103">
+      <c r="D103" s="2">
         <v>0.32</v>
       </c>
-      <c r="F103">
+      <c r="F103" s="2">
         <v>300000</v>
       </c>
-      <c r="H103">
+      <c r="H103" s="2">
         <v>6</v>
       </c>
-      <c r="I103" t="s">
+      <c r="I103" s="2" t="s">
         <v>244</v>
       </c>
-      <c r="L103" t="s">
+      <c r="L103" s="2" t="s">
         <v>184</v>
       </c>
-      <c r="M103" t="s">
+      <c r="M103" s="2" t="s">
         <v>24</v>
       </c>
-      <c r="N103" t="s">
+      <c r="N103" s="2" t="s">
         <v>25</v>
       </c>
-      <c r="O103" t="s">
-        <v>26</v>
-      </c>
-      <c r="P103" t="s">
+      <c r="O103" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="P103" s="2" t="s">
         <v>239</v>
       </c>
-      <c r="Q103" t="s">
+      <c r="Q103" s="2" t="s">
         <v>240</v>
       </c>
-      <c r="T103" t="s">
+      <c r="T103" s="2" t="s">
         <v>101</v>
       </c>
-      <c r="U103" t="s">
+      <c r="U103" s="2" t="s">
         <v>241</v>
       </c>
     </row>
-    <row r="104" spans="1:21" x14ac:dyDescent="0.3">
-      <c r="A104" t="s">
+    <row r="104" spans="1:21" s="2" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A104" s="2" t="s">
         <v>249</v>
       </c>
-      <c r="B104" t="s">
+      <c r="B104" s="2" t="s">
         <v>250</v>
       </c>
-      <c r="C104">
+      <c r="C104" s="2">
         <v>3</v>
       </c>
-      <c r="D104">
+      <c r="D104" s="2">
         <v>0.32</v>
       </c>
-      <c r="F104">
+      <c r="F104" s="2">
         <v>300000</v>
       </c>
-      <c r="H104">
+      <c r="H104" s="2">
         <v>8</v>
       </c>
-      <c r="I104" t="s">
+      <c r="I104" s="2" t="s">
         <v>251</v>
       </c>
-      <c r="L104" t="s">
+      <c r="L104" s="2" t="s">
         <v>184</v>
       </c>
-      <c r="M104" t="s">
+      <c r="M104" s="2" t="s">
         <v>24</v>
       </c>
-      <c r="N104" t="s">
+      <c r="N104" s="2" t="s">
         <v>25</v>
       </c>
-      <c r="O104" t="s">
-        <v>26</v>
-      </c>
-      <c r="P104" t="s">
+      <c r="O104" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="P104" s="2" t="s">
         <v>239</v>
       </c>
-      <c r="Q104" t="s">
+      <c r="Q104" s="2" t="s">
         <v>240</v>
       </c>
-      <c r="T104" t="s">
+      <c r="T104" s="2" t="s">
         <v>101</v>
       </c>
-      <c r="U104" t="s">
+      <c r="U104" s="2" t="s">
         <v>241</v>
       </c>
     </row>
-    <row r="105" spans="1:21" x14ac:dyDescent="0.3">
-      <c r="A105" t="s">
+    <row r="105" spans="1:21" s="2" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A105" s="2" t="s">
         <v>252</v>
       </c>
-      <c r="B105" t="s">
+      <c r="B105" s="2" t="s">
         <v>253</v>
       </c>
-      <c r="C105">
+      <c r="C105" s="2">
         <v>3</v>
       </c>
-      <c r="D105">
+      <c r="D105" s="2">
         <v>0.32</v>
       </c>
-      <c r="F105">
+      <c r="F105" s="2">
         <v>300000</v>
       </c>
-      <c r="H105">
+      <c r="H105" s="2">
         <v>8</v>
       </c>
-      <c r="I105" t="s">
+      <c r="I105" s="2" t="s">
         <v>244</v>
       </c>
-      <c r="L105" t="s">
+      <c r="L105" s="2" t="s">
         <v>184</v>
       </c>
-      <c r="M105" t="s">
+      <c r="M105" s="2" t="s">
         <v>24</v>
       </c>
-      <c r="N105" t="s">
+      <c r="N105" s="2" t="s">
         <v>25</v>
       </c>
-      <c r="O105" t="s">
-        <v>26</v>
-      </c>
-      <c r="P105" t="s">
+      <c r="O105" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="P105" s="2" t="s">
         <v>239</v>
       </c>
-      <c r="Q105" t="s">
+      <c r="Q105" s="2" t="s">
         <v>240</v>
       </c>
-      <c r="T105" t="s">
+      <c r="T105" s="2" t="s">
         <v>101</v>
       </c>
-      <c r="U105" t="s">
+      <c r="U105" s="2" t="s">
         <v>241</v>
       </c>
     </row>
-    <row r="106" spans="1:21" x14ac:dyDescent="0.3">
-      <c r="A106" t="s">
+    <row r="106" spans="1:21" s="2" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A106" s="2" t="s">
         <v>254</v>
       </c>
-      <c r="B106" t="s">
+      <c r="B106" s="2" t="s">
         <v>255</v>
       </c>
-      <c r="C106">
+      <c r="C106" s="2">
         <v>3</v>
       </c>
-      <c r="D106">
+      <c r="D106" s="2">
         <v>0.32</v>
       </c>
-      <c r="F106">
+      <c r="F106" s="2">
         <v>300000</v>
       </c>
-      <c r="H106">
+      <c r="H106" s="2">
         <v>10</v>
       </c>
-      <c r="I106" t="s">
+      <c r="I106" s="2" t="s">
         <v>244</v>
       </c>
-      <c r="L106" t="s">
+      <c r="L106" s="2" t="s">
         <v>184</v>
       </c>
-      <c r="M106" t="s">
+      <c r="M106" s="2" t="s">
         <v>24</v>
       </c>
-      <c r="N106" t="s">
+      <c r="N106" s="2" t="s">
         <v>25</v>
       </c>
-      <c r="O106" t="s">
-        <v>26</v>
-      </c>
-      <c r="P106" t="s">
+      <c r="O106" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="P106" s="2" t="s">
         <v>239</v>
       </c>
-      <c r="Q106" t="s">
+      <c r="Q106" s="2" t="s">
         <v>240</v>
       </c>
-      <c r="T106" t="s">
+      <c r="T106" s="2" t="s">
         <v>101</v>
       </c>
-      <c r="U106" t="s">
+      <c r="U106" s="2" t="s">
         <v>241</v>
       </c>
     </row>
-    <row r="107" spans="1:21" x14ac:dyDescent="0.3">
-      <c r="A107" t="s">
+    <row r="107" spans="1:21" s="2" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A107" s="2" t="s">
         <v>256</v>
       </c>
-      <c r="B107" t="s">
+      <c r="B107" s="2" t="s">
         <v>257</v>
       </c>
-      <c r="C107">
+      <c r="C107" s="2">
         <v>3</v>
       </c>
-      <c r="D107">
+      <c r="D107" s="2">
         <v>0.32</v>
       </c>
-      <c r="F107">
+      <c r="F107" s="2">
         <v>300000</v>
       </c>
-      <c r="H107">
+      <c r="H107" s="2">
         <v>12</v>
       </c>
-      <c r="I107" t="s">
+      <c r="I107" s="2" t="s">
         <v>244</v>
       </c>
-      <c r="L107" t="s">
+      <c r="L107" s="2" t="s">
         <v>184</v>
       </c>
-      <c r="M107" t="s">
+      <c r="M107" s="2" t="s">
         <v>24</v>
       </c>
-      <c r="N107" t="s">
+      <c r="N107" s="2" t="s">
         <v>25</v>
       </c>
-      <c r="O107" t="s">
-        <v>26</v>
-      </c>
-      <c r="P107" t="s">
+      <c r="O107" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="P107" s="2" t="s">
         <v>239</v>
       </c>
-      <c r="Q107" t="s">
+      <c r="Q107" s="2" t="s">
         <v>240</v>
       </c>
-      <c r="T107" t="s">
+      <c r="T107" s="2" t="s">
         <v>101</v>
       </c>
-      <c r="U107" t="s">
+      <c r="U107" s="2" t="s">
         <v>241</v>
       </c>
     </row>
-    <row r="108" spans="1:21" x14ac:dyDescent="0.3">
-      <c r="A108" t="s">
+    <row r="108" spans="1:21" s="2" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A108" s="2" t="s">
         <v>258</v>
       </c>
-      <c r="B108" t="s">
+      <c r="B108" s="2" t="s">
         <v>259</v>
       </c>
-      <c r="C108">
+      <c r="C108" s="2">
         <v>3</v>
       </c>
-      <c r="D108">
+      <c r="D108" s="2">
         <v>0.32</v>
       </c>
-      <c r="F108">
+      <c r="F108" s="2">
         <v>300000</v>
       </c>
-      <c r="H108">
+      <c r="H108" s="2">
         <v>16</v>
       </c>
-      <c r="I108" t="s">
+      <c r="I108" s="2" t="s">
         <v>244</v>
       </c>
-      <c r="L108" t="s">
+      <c r="L108" s="2" t="s">
         <v>184</v>
       </c>
-      <c r="M108" t="s">
+      <c r="M108" s="2" t="s">
         <v>24</v>
       </c>
-      <c r="N108" t="s">
+      <c r="N108" s="2" t="s">
         <v>25</v>
       </c>
-      <c r="O108" t="s">
-        <v>26</v>
-      </c>
-      <c r="P108" t="s">
+      <c r="O108" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="P108" s="2" t="s">
         <v>239</v>
       </c>
-      <c r="Q108" t="s">
+      <c r="Q108" s="2" t="s">
         <v>240</v>
       </c>
-      <c r="T108" t="s">
+      <c r="T108" s="2" t="s">
         <v>101</v>
       </c>
-      <c r="U108" t="s">
+      <c r="U108" s="2" t="s">
         <v>241</v>
       </c>
     </row>
-    <row r="109" spans="1:21" x14ac:dyDescent="0.3">
-      <c r="A109" t="s">
+    <row r="109" spans="1:21" s="2" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A109" s="2" t="s">
         <v>260</v>
       </c>
-      <c r="B109" t="s">
+      <c r="B109" s="2" t="s">
         <v>261</v>
       </c>
-      <c r="C109">
+      <c r="C109" s="2">
         <v>3</v>
       </c>
-      <c r="D109">
+      <c r="D109" s="2">
         <v>0.32</v>
       </c>
-      <c r="F109">
+      <c r="F109" s="2">
         <v>400000</v>
       </c>
-      <c r="H109">
+      <c r="H109" s="2">
         <v>0</v>
       </c>
-      <c r="L109" t="s">
+      <c r="L109" s="2" t="s">
         <v>184</v>
       </c>
-      <c r="M109" t="s">
+      <c r="M109" s="2" t="s">
         <v>24</v>
       </c>
-      <c r="N109" t="s">
+      <c r="N109" s="2" t="s">
         <v>25</v>
       </c>
-      <c r="O109" t="s">
-        <v>26</v>
-      </c>
-      <c r="P109" t="s">
+      <c r="O109" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="P109" s="2" t="s">
         <v>239</v>
       </c>
-      <c r="Q109" t="s">
+      <c r="Q109" s="2" t="s">
         <v>240</v>
       </c>
-      <c r="T109" t="s">
+      <c r="T109" s="2" t="s">
         <v>101</v>
       </c>
-      <c r="U109" t="s">
+      <c r="U109" s="2" t="s">
         <v>241</v>
       </c>
     </row>
-    <row r="110" spans="1:21" x14ac:dyDescent="0.3">
-      <c r="A110" t="s">
+    <row r="110" spans="1:21" s="2" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A110" s="2" t="s">
         <v>262</v>
       </c>
-      <c r="B110" t="s">
+      <c r="B110" s="2" t="s">
         <v>263</v>
       </c>
-      <c r="C110">
+      <c r="C110" s="2">
         <v>3</v>
       </c>
-      <c r="D110">
+      <c r="D110" s="2">
         <v>0.32</v>
       </c>
-      <c r="F110">
+      <c r="F110" s="2">
         <v>400000</v>
       </c>
-      <c r="H110">
+      <c r="H110" s="2">
         <v>2</v>
       </c>
-      <c r="I110" t="s">
+      <c r="I110" s="2" t="s">
         <v>244</v>
       </c>
-      <c r="L110" t="s">
+      <c r="L110" s="2" t="s">
         <v>184</v>
       </c>
-      <c r="M110" t="s">
+      <c r="M110" s="2" t="s">
         <v>24</v>
       </c>
-      <c r="N110" t="s">
+      <c r="N110" s="2" t="s">
         <v>25</v>
       </c>
-      <c r="O110" t="s">
-        <v>26</v>
-      </c>
-      <c r="P110" t="s">
+      <c r="O110" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="P110" s="2" t="s">
         <v>239</v>
       </c>
-      <c r="Q110" t="s">
+      <c r="Q110" s="2" t="s">
         <v>240</v>
       </c>
-      <c r="T110" t="s">
+      <c r="T110" s="2" t="s">
         <v>101</v>
       </c>
-      <c r="U110" t="s">
+      <c r="U110" s="2" t="s">
         <v>241</v>
       </c>
     </row>
-    <row r="111" spans="1:21" x14ac:dyDescent="0.3">
-      <c r="A111" t="s">
+    <row r="111" spans="1:21" s="2" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A111" s="2" t="s">
         <v>264</v>
       </c>
-      <c r="B111" t="s">
+      <c r="B111" s="2" t="s">
         <v>265</v>
       </c>
-      <c r="C111">
+      <c r="C111" s="2">
         <v>3</v>
       </c>
-      <c r="D111">
+      <c r="D111" s="2">
         <v>0.32</v>
       </c>
-      <c r="F111">
+      <c r="F111" s="2">
         <v>400000</v>
       </c>
-      <c r="H111">
+      <c r="H111" s="2">
         <v>4</v>
       </c>
-      <c r="I111" t="s">
+      <c r="I111" s="2" t="s">
         <v>244</v>
       </c>
-      <c r="L111" t="s">
+      <c r="L111" s="2" t="s">
         <v>184</v>
       </c>
-      <c r="M111" t="s">
+      <c r="M111" s="2" t="s">
         <v>24</v>
       </c>
-      <c r="N111" t="s">
+      <c r="N111" s="2" t="s">
         <v>25</v>
       </c>
-      <c r="O111" t="s">
-        <v>26</v>
-      </c>
-      <c r="P111" t="s">
+      <c r="O111" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="P111" s="2" t="s">
         <v>239</v>
       </c>
-      <c r="Q111" t="s">
+      <c r="Q111" s="2" t="s">
         <v>240</v>
       </c>
-      <c r="T111" t="s">
+      <c r="T111" s="2" t="s">
         <v>101</v>
       </c>
-      <c r="U111" t="s">
+      <c r="U111" s="2" t="s">
         <v>241</v>
       </c>
     </row>
-    <row r="112" spans="1:21" x14ac:dyDescent="0.3">
-      <c r="A112" t="s">
+    <row r="112" spans="1:21" s="2" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A112" s="2" t="s">
         <v>266</v>
       </c>
-      <c r="B112" t="s">
+      <c r="B112" s="2" t="s">
         <v>267</v>
       </c>
-      <c r="C112">
+      <c r="C112" s="2">
         <v>3</v>
       </c>
-      <c r="D112">
+      <c r="D112" s="2">
         <v>0.32</v>
       </c>
-      <c r="F112">
+      <c r="F112" s="2">
         <v>400000</v>
       </c>
-      <c r="H112">
+      <c r="H112" s="2">
         <v>6</v>
       </c>
-      <c r="I112" t="s">
+      <c r="I112" s="2" t="s">
         <v>244</v>
       </c>
-      <c r="L112" t="s">
+      <c r="L112" s="2" t="s">
         <v>184</v>
       </c>
-      <c r="M112" t="s">
+      <c r="M112" s="2" t="s">
         <v>24</v>
       </c>
-      <c r="N112" t="s">
+      <c r="N112" s="2" t="s">
         <v>25</v>
       </c>
-      <c r="O112" t="s">
-        <v>26</v>
-      </c>
-      <c r="P112" t="s">
+      <c r="O112" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="P112" s="2" t="s">
         <v>239</v>
       </c>
-      <c r="Q112" t="s">
+      <c r="Q112" s="2" t="s">
         <v>240</v>
       </c>
-      <c r="T112" t="s">
+      <c r="T112" s="2" t="s">
         <v>101</v>
       </c>
-      <c r="U112" t="s">
+      <c r="U112" s="2" t="s">
         <v>241</v>
       </c>
     </row>
-    <row r="113" spans="1:21" x14ac:dyDescent="0.3">
-      <c r="A113" t="s">
+    <row r="113" spans="1:21" s="2" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A113" s="2" t="s">
         <v>268</v>
       </c>
-      <c r="B113" t="s">
+      <c r="B113" s="2" t="s">
         <v>269</v>
       </c>
-      <c r="C113">
+      <c r="C113" s="2">
         <v>3</v>
       </c>
-      <c r="D113">
+      <c r="D113" s="2">
         <v>0.32</v>
       </c>
-      <c r="F113">
+      <c r="F113" s="2">
         <v>400000</v>
       </c>
-      <c r="H113">
+      <c r="H113" s="2">
         <v>8</v>
       </c>
-      <c r="I113" t="s">
+      <c r="I113" s="2" t="s">
         <v>251</v>
       </c>
-      <c r="L113" t="s">
+      <c r="L113" s="2" t="s">
         <v>184</v>
       </c>
-      <c r="M113" t="s">
+      <c r="M113" s="2" t="s">
         <v>24</v>
       </c>
-      <c r="N113" t="s">
+      <c r="N113" s="2" t="s">
         <v>25</v>
       </c>
-      <c r="O113" t="s">
-        <v>26</v>
-      </c>
-      <c r="P113" t="s">
+      <c r="O113" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="P113" s="2" t="s">
         <v>239</v>
       </c>
-      <c r="Q113" t="s">
+      <c r="Q113" s="2" t="s">
         <v>240</v>
       </c>
-      <c r="T113" t="s">
+      <c r="T113" s="2" t="s">
         <v>101</v>
       </c>
-      <c r="U113" t="s">
+      <c r="U113" s="2" t="s">
         <v>241</v>
       </c>
     </row>
-    <row r="114" spans="1:21" x14ac:dyDescent="0.3">
-      <c r="A114" t="s">
+    <row r="114" spans="1:21" s="2" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A114" s="2" t="s">
         <v>270</v>
       </c>
-      <c r="B114" t="s">
+      <c r="B114" s="2" t="s">
         <v>271</v>
       </c>
-      <c r="C114">
+      <c r="C114" s="2">
         <v>3</v>
       </c>
-      <c r="D114">
+      <c r="D114" s="2">
         <v>0.32</v>
       </c>
-      <c r="F114">
+      <c r="F114" s="2">
         <v>400000</v>
       </c>
-      <c r="H114">
+      <c r="H114" s="2">
         <v>8</v>
       </c>
-      <c r="I114" t="s">
+      <c r="I114" s="2" t="s">
         <v>244</v>
       </c>
-      <c r="L114" t="s">
+      <c r="L114" s="2" t="s">
         <v>184</v>
       </c>
-      <c r="M114" t="s">
+      <c r="M114" s="2" t="s">
         <v>24</v>
       </c>
-      <c r="N114" t="s">
+      <c r="N114" s="2" t="s">
         <v>25</v>
       </c>
-      <c r="O114" t="s">
-        <v>26</v>
-      </c>
-      <c r="P114" t="s">
+      <c r="O114" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="P114" s="2" t="s">
         <v>239</v>
       </c>
-      <c r="Q114" t="s">
+      <c r="Q114" s="2" t="s">
         <v>240</v>
       </c>
-      <c r="T114" t="s">
+      <c r="T114" s="2" t="s">
         <v>101</v>
       </c>
-      <c r="U114" t="s">
+      <c r="U114" s="2" t="s">
         <v>241</v>
       </c>
     </row>
-    <row r="115" spans="1:21" x14ac:dyDescent="0.3">
-      <c r="A115" t="s">
+    <row r="115" spans="1:21" s="2" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A115" s="2" t="s">
         <v>272</v>
       </c>
-      <c r="B115" t="s">
+      <c r="B115" s="2" t="s">
         <v>273</v>
       </c>
-      <c r="C115">
+      <c r="C115" s="2">
         <v>3</v>
       </c>
-      <c r="D115">
+      <c r="D115" s="2">
         <v>0.32</v>
       </c>
-      <c r="F115">
+      <c r="F115" s="2">
         <v>400000</v>
       </c>
-      <c r="H115">
+      <c r="H115" s="2">
         <v>10</v>
       </c>
-      <c r="I115" t="s">
+      <c r="I115" s="2" t="s">
         <v>244</v>
       </c>
-      <c r="L115" t="s">
+      <c r="L115" s="2" t="s">
         <v>184</v>
       </c>
-      <c r="M115" t="s">
+      <c r="M115" s="2" t="s">
         <v>24</v>
       </c>
-      <c r="N115" t="s">
+      <c r="N115" s="2" t="s">
         <v>25</v>
       </c>
-      <c r="O115" t="s">
-        <v>26</v>
-      </c>
-      <c r="P115" t="s">
+      <c r="O115" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="P115" s="2" t="s">
         <v>239</v>
       </c>
-      <c r="Q115" t="s">
+      <c r="Q115" s="2" t="s">
         <v>240</v>
       </c>
-      <c r="T115" t="s">
+      <c r="T115" s="2" t="s">
         <v>101</v>
       </c>
-      <c r="U115" t="s">
+      <c r="U115" s="2" t="s">
         <v>241</v>
       </c>
     </row>
-    <row r="116" spans="1:21" x14ac:dyDescent="0.3">
-      <c r="A116" t="s">
+    <row r="116" spans="1:21" s="2" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A116" s="2" t="s">
         <v>274</v>
       </c>
-      <c r="B116" t="s">
+      <c r="B116" s="2" t="s">
         <v>275</v>
       </c>
-      <c r="C116">
+      <c r="C116" s="2">
         <v>3</v>
       </c>
-      <c r="D116">
+      <c r="D116" s="2">
         <v>0.32</v>
       </c>
-      <c r="F116">
+      <c r="F116" s="2">
         <v>400000</v>
       </c>
-      <c r="H116">
+      <c r="H116" s="2">
         <v>12</v>
       </c>
-      <c r="I116" t="s">
+      <c r="I116" s="2" t="s">
         <v>244</v>
       </c>
-      <c r="L116" t="s">
+      <c r="L116" s="2" t="s">
         <v>184</v>
       </c>
-      <c r="M116" t="s">
+      <c r="M116" s="2" t="s">
         <v>24</v>
       </c>
-      <c r="N116" t="s">
+      <c r="N116" s="2" t="s">
         <v>25</v>
       </c>
-      <c r="O116" t="s">
-        <v>26</v>
-      </c>
-      <c r="P116" t="s">
+      <c r="O116" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="P116" s="2" t="s">
         <v>239</v>
       </c>
-      <c r="Q116" t="s">
+      <c r="Q116" s="2" t="s">
         <v>240</v>
       </c>
-      <c r="T116" t="s">
+      <c r="T116" s="2" t="s">
         <v>101</v>
       </c>
-      <c r="U116" t="s">
+      <c r="U116" s="2" t="s">
         <v>241</v>
       </c>
     </row>
-    <row r="117" spans="1:21" x14ac:dyDescent="0.3">
-      <c r="A117" t="s">
+    <row r="117" spans="1:21" s="2" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A117" s="2" t="s">
         <v>276</v>
       </c>
-      <c r="B117" t="s">
+      <c r="B117" s="2" t="s">
         <v>277</v>
       </c>
-      <c r="C117">
+      <c r="C117" s="2">
         <v>3</v>
       </c>
-      <c r="D117">
+      <c r="D117" s="2">
         <v>0.32</v>
       </c>
-      <c r="F117">
+      <c r="F117" s="2">
         <v>400000</v>
       </c>
-      <c r="H117">
+      <c r="H117" s="2">
         <v>16</v>
       </c>
-      <c r="I117" t="s">
+      <c r="I117" s="2" t="s">
         <v>244</v>
       </c>
-      <c r="L117" t="s">
+      <c r="L117" s="2" t="s">
         <v>184</v>
       </c>
-      <c r="M117" t="s">
+      <c r="M117" s="2" t="s">
         <v>24</v>
       </c>
-      <c r="N117" t="s">
+      <c r="N117" s="2" t="s">
         <v>25</v>
       </c>
-      <c r="O117" t="s">
-        <v>26</v>
-      </c>
-      <c r="P117" t="s">
+      <c r="O117" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="P117" s="2" t="s">
         <v>239</v>
       </c>
-      <c r="Q117" t="s">
+      <c r="Q117" s="2" t="s">
         <v>240</v>
       </c>
-      <c r="T117" t="s">
+      <c r="T117" s="2" t="s">
         <v>101</v>
       </c>
-      <c r="U117" t="s">
+      <c r="U117" s="2" t="s">
         <v>241</v>
       </c>
     </row>
-    <row r="118" spans="1:21" x14ac:dyDescent="0.3">
-      <c r="A118" t="s">
+    <row r="118" spans="1:21" s="2" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A118" s="2" t="s">
         <v>278</v>
       </c>
-      <c r="B118" t="s">
+      <c r="B118" s="2" t="s">
         <v>279</v>
       </c>
-      <c r="C118">
+      <c r="C118" s="2">
         <v>3</v>
       </c>
-      <c r="D118">
+      <c r="D118" s="2">
         <v>0.32</v>
       </c>
-      <c r="F118">
+      <c r="F118" s="2">
         <v>500000</v>
       </c>
-      <c r="H118">
+      <c r="H118" s="2">
         <v>0</v>
       </c>
-      <c r="L118" t="s">
+      <c r="L118" s="2" t="s">
         <v>184</v>
       </c>
-      <c r="M118" t="s">
+      <c r="M118" s="2" t="s">
         <v>24</v>
       </c>
-      <c r="N118" t="s">
+      <c r="N118" s="2" t="s">
         <v>25</v>
       </c>
-      <c r="O118" t="s">
-        <v>26</v>
-      </c>
-      <c r="P118" t="s">
+      <c r="O118" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="P118" s="2" t="s">
         <v>239</v>
       </c>
-      <c r="Q118" t="s">
+      <c r="Q118" s="2" t="s">
         <v>240</v>
       </c>
-      <c r="T118" t="s">
+      <c r="T118" s="2" t="s">
         <v>101</v>
       </c>
-      <c r="U118" t="s">
+      <c r="U118" s="2" t="s">
         <v>241</v>
       </c>
     </row>
-    <row r="119" spans="1:21" x14ac:dyDescent="0.3">
-      <c r="A119" t="s">
+    <row r="119" spans="1:21" s="2" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A119" s="2" t="s">
         <v>280</v>
       </c>
-      <c r="B119" t="s">
+      <c r="B119" s="2" t="s">
         <v>281</v>
       </c>
-      <c r="C119">
+      <c r="C119" s="2">
         <v>3</v>
       </c>
-      <c r="D119">
+      <c r="D119" s="2">
         <v>0.32</v>
       </c>
-      <c r="F119">
+      <c r="F119" s="2">
         <v>500000</v>
       </c>
-      <c r="H119">
+      <c r="H119" s="2">
         <v>2</v>
       </c>
-      <c r="I119" t="s">
+      <c r="I119" s="2" t="s">
         <v>244</v>
       </c>
-      <c r="L119" t="s">
+      <c r="L119" s="2" t="s">
         <v>184</v>
       </c>
-      <c r="M119" t="s">
+      <c r="M119" s="2" t="s">
         <v>24</v>
       </c>
-      <c r="N119" t="s">
+      <c r="N119" s="2" t="s">
         <v>25</v>
       </c>
-      <c r="O119" t="s">
-        <v>26</v>
-      </c>
-      <c r="P119" t="s">
+      <c r="O119" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="P119" s="2" t="s">
         <v>239</v>
       </c>
-      <c r="Q119" t="s">
+      <c r="Q119" s="2" t="s">
         <v>240</v>
       </c>
-      <c r="T119" t="s">
+      <c r="T119" s="2" t="s">
         <v>101</v>
       </c>
-      <c r="U119" t="s">
+      <c r="U119" s="2" t="s">
         <v>241</v>
       </c>
     </row>
-    <row r="120" spans="1:21" x14ac:dyDescent="0.3">
-      <c r="A120" t="s">
+    <row r="120" spans="1:21" s="2" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A120" s="2" t="s">
         <v>282</v>
       </c>
-      <c r="B120" t="s">
+      <c r="B120" s="2" t="s">
         <v>283</v>
       </c>
-      <c r="C120">
+      <c r="C120" s="2">
         <v>3</v>
       </c>
-      <c r="D120">
+      <c r="D120" s="2">
         <v>0.32</v>
       </c>
-      <c r="F120">
+      <c r="F120" s="2">
         <v>500000</v>
       </c>
-      <c r="H120">
+      <c r="H120" s="2">
         <v>4</v>
       </c>
-      <c r="I120" t="s">
+      <c r="I120" s="2" t="s">
         <v>244</v>
       </c>
-      <c r="L120" t="s">
+      <c r="L120" s="2" t="s">
         <v>184</v>
       </c>
-      <c r="M120" t="s">
+      <c r="M120" s="2" t="s">
         <v>24</v>
       </c>
-      <c r="N120" t="s">
+      <c r="N120" s="2" t="s">
         <v>25</v>
       </c>
-      <c r="O120" t="s">
-        <v>26</v>
-      </c>
-      <c r="P120" t="s">
+      <c r="O120" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="P120" s="2" t="s">
         <v>239</v>
       </c>
-      <c r="Q120" t="s">
+      <c r="Q120" s="2" t="s">
         <v>240</v>
       </c>
-      <c r="T120" t="s">
+      <c r="T120" s="2" t="s">
         <v>101</v>
       </c>
-      <c r="U120" t="s">
+      <c r="U120" s="2" t="s">
         <v>241</v>
       </c>
     </row>
-    <row r="121" spans="1:21" x14ac:dyDescent="0.3">
-      <c r="A121" t="s">
+    <row r="121" spans="1:21" s="2" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A121" s="2" t="s">
         <v>284</v>
       </c>
-      <c r="B121" t="s">
+      <c r="B121" s="2" t="s">
         <v>285</v>
       </c>
-      <c r="C121">
+      <c r="C121" s="2">
         <v>3</v>
       </c>
-      <c r="D121">
+      <c r="D121" s="2">
         <v>0.32</v>
       </c>
-      <c r="F121">
+      <c r="F121" s="2">
         <v>500000</v>
       </c>
-      <c r="H121">
+      <c r="H121" s="2">
         <v>6</v>
       </c>
-      <c r="I121" t="s">
+      <c r="I121" s="2" t="s">
         <v>244</v>
       </c>
-      <c r="L121" t="s">
+      <c r="L121" s="2" t="s">
         <v>184</v>
       </c>
-      <c r="M121" t="s">
+      <c r="M121" s="2" t="s">
         <v>24</v>
       </c>
-      <c r="N121" t="s">
+      <c r="N121" s="2" t="s">
         <v>25</v>
       </c>
-      <c r="O121" t="s">
-        <v>26</v>
-      </c>
-      <c r="P121" t="s">
+      <c r="O121" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="P121" s="2" t="s">
         <v>239</v>
       </c>
-      <c r="Q121" t="s">
+      <c r="Q121" s="2" t="s">
         <v>240</v>
       </c>
-      <c r="T121" t="s">
+      <c r="T121" s="2" t="s">
         <v>101</v>
       </c>
-      <c r="U121" t="s">
+      <c r="U121" s="2" t="s">
         <v>241</v>
       </c>
     </row>
-    <row r="122" spans="1:21" x14ac:dyDescent="0.3">
-      <c r="A122" t="s">
+    <row r="122" spans="1:21" s="2" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A122" s="2" t="s">
         <v>286</v>
       </c>
-      <c r="B122" t="s">
+      <c r="B122" s="2" t="s">
         <v>287</v>
       </c>
-      <c r="C122">
+      <c r="C122" s="2">
         <v>3</v>
       </c>
-      <c r="D122">
+      <c r="D122" s="2">
         <v>0.32</v>
       </c>
-      <c r="F122">
+      <c r="F122" s="2">
         <v>500000</v>
       </c>
-      <c r="H122">
+      <c r="H122" s="2">
         <v>8</v>
       </c>
-      <c r="I122" t="s">
+      <c r="I122" s="2" t="s">
         <v>251</v>
       </c>
-      <c r="L122" t="s">
+      <c r="L122" s="2" t="s">
         <v>184</v>
       </c>
-      <c r="M122" t="s">
+      <c r="M122" s="2" t="s">
         <v>24</v>
       </c>
-      <c r="N122" t="s">
+      <c r="N122" s="2" t="s">
         <v>25</v>
       </c>
-      <c r="O122" t="s">
-        <v>26</v>
-      </c>
-      <c r="P122" t="s">
+      <c r="O122" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="P122" s="2" t="s">
         <v>239</v>
       </c>
-      <c r="Q122" t="s">
+      <c r="Q122" s="2" t="s">
         <v>240</v>
       </c>
-      <c r="T122" t="s">
+      <c r="T122" s="2" t="s">
         <v>101</v>
       </c>
-      <c r="U122" t="s">
+      <c r="U122" s="2" t="s">
         <v>241</v>
       </c>
     </row>
-    <row r="123" spans="1:21" x14ac:dyDescent="0.3">
-      <c r="A123" t="s">
+    <row r="123" spans="1:21" s="2" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A123" s="2" t="s">
         <v>288</v>
       </c>
-      <c r="B123" t="s">
+      <c r="B123" s="2" t="s">
         <v>289</v>
       </c>
-      <c r="C123">
+      <c r="C123" s="2">
         <v>3</v>
       </c>
-      <c r="D123">
+      <c r="D123" s="2">
         <v>0.32</v>
       </c>
-      <c r="F123">
+      <c r="F123" s="2">
         <v>500000</v>
       </c>
-      <c r="H123">
+      <c r="H123" s="2">
         <v>8</v>
       </c>
-      <c r="I123" t="s">
+      <c r="I123" s="2" t="s">
         <v>244</v>
       </c>
-      <c r="L123" t="s">
+      <c r="L123" s="2" t="s">
         <v>184</v>
       </c>
-      <c r="M123" t="s">
+      <c r="M123" s="2" t="s">
         <v>24</v>
       </c>
-      <c r="N123" t="s">
+      <c r="N123" s="2" t="s">
         <v>25</v>
       </c>
-      <c r="O123" t="s">
-        <v>26</v>
-      </c>
-      <c r="P123" t="s">
+      <c r="O123" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="P123" s="2" t="s">
         <v>239</v>
       </c>
-      <c r="Q123" t="s">
+      <c r="Q123" s="2" t="s">
         <v>240</v>
       </c>
-      <c r="T123" t="s">
+      <c r="T123" s="2" t="s">
         <v>101</v>
       </c>
-      <c r="U123" t="s">
+      <c r="U123" s="2" t="s">
         <v>241</v>
       </c>
     </row>
-    <row r="124" spans="1:21" x14ac:dyDescent="0.3">
-      <c r="A124" t="s">
+    <row r="124" spans="1:21" s="2" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A124" s="2" t="s">
         <v>290</v>
       </c>
-      <c r="B124" t="s">
+      <c r="B124" s="2" t="s">
         <v>291</v>
       </c>
-      <c r="C124">
+      <c r="C124" s="2">
         <v>3</v>
       </c>
-      <c r="D124">
+      <c r="D124" s="2">
         <v>0.32</v>
       </c>
-      <c r="F124">
+      <c r="F124" s="2">
         <v>500000</v>
       </c>
-      <c r="H124">
+      <c r="H124" s="2">
         <v>10</v>
       </c>
-      <c r="I124" t="s">
+      <c r="I124" s="2" t="s">
         <v>244</v>
       </c>
-      <c r="L124" t="s">
+      <c r="L124" s="2" t="s">
         <v>184</v>
       </c>
-      <c r="M124" t="s">
+      <c r="M124" s="2" t="s">
         <v>24</v>
       </c>
-      <c r="N124" t="s">
+      <c r="N124" s="2" t="s">
         <v>25</v>
       </c>
-      <c r="O124" t="s">
-        <v>26</v>
-      </c>
-      <c r="P124" t="s">
+      <c r="O124" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="P124" s="2" t="s">
         <v>239</v>
       </c>
-      <c r="Q124" t="s">
+      <c r="Q124" s="2" t="s">
         <v>240</v>
       </c>
-      <c r="T124" t="s">
+      <c r="T124" s="2" t="s">
         <v>101</v>
       </c>
-      <c r="U124" t="s">
+      <c r="U124" s="2" t="s">
         <v>241</v>
       </c>
     </row>
-    <row r="125" spans="1:21" x14ac:dyDescent="0.3">
-      <c r="A125" t="s">
+    <row r="125" spans="1:21" s="2" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A125" s="2" t="s">
         <v>292</v>
       </c>
-      <c r="B125" t="s">
+      <c r="B125" s="2" t="s">
         <v>293</v>
       </c>
-      <c r="C125">
+      <c r="C125" s="2">
         <v>3</v>
       </c>
-      <c r="D125">
+      <c r="D125" s="2">
         <v>0.32</v>
       </c>
-      <c r="F125">
+      <c r="F125" s="2">
         <v>500000</v>
       </c>
-      <c r="H125">
+      <c r="H125" s="2">
         <v>12</v>
       </c>
-      <c r="I125" t="s">
+      <c r="I125" s="2" t="s">
         <v>244</v>
       </c>
-      <c r="L125" t="s">
+      <c r="L125" s="2" t="s">
         <v>184</v>
       </c>
-      <c r="M125" t="s">
+      <c r="M125" s="2" t="s">
         <v>24</v>
       </c>
-      <c r="N125" t="s">
+      <c r="N125" s="2" t="s">
         <v>25</v>
       </c>
-      <c r="O125" t="s">
-        <v>26</v>
-      </c>
-      <c r="P125" t="s">
+      <c r="O125" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="P125" s="2" t="s">
         <v>239</v>
       </c>
-      <c r="Q125" t="s">
+      <c r="Q125" s="2" t="s">
         <v>240</v>
       </c>
-      <c r="T125" t="s">
+      <c r="T125" s="2" t="s">
         <v>101</v>
       </c>
-      <c r="U125" t="s">
+      <c r="U125" s="2" t="s">
         <v>241</v>
       </c>
     </row>
-    <row r="126" spans="1:21" x14ac:dyDescent="0.3">
-      <c r="A126" t="s">
+    <row r="126" spans="1:21" s="2" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A126" s="2" t="s">
         <v>294</v>
       </c>
-      <c r="B126" t="s">
+      <c r="B126" s="2" t="s">
         <v>295</v>
       </c>
-      <c r="C126">
+      <c r="C126" s="2">
         <v>3</v>
       </c>
-      <c r="D126">
+      <c r="D126" s="2">
         <v>0.32</v>
       </c>
-      <c r="F126">
+      <c r="F126" s="2">
         <v>500000</v>
       </c>
-      <c r="H126">
+      <c r="H126" s="2">
         <v>16</v>
       </c>
-      <c r="I126" t="s">
+      <c r="I126" s="2" t="s">
         <v>244</v>
       </c>
-      <c r="L126" t="s">
+      <c r="L126" s="2" t="s">
         <v>184</v>
       </c>
-      <c r="M126" t="s">
+      <c r="M126" s="2" t="s">
         <v>24</v>
       </c>
-      <c r="N126" t="s">
+      <c r="N126" s="2" t="s">
         <v>25</v>
       </c>
-      <c r="O126" t="s">
-        <v>26</v>
-      </c>
-      <c r="P126" t="s">
+      <c r="O126" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="P126" s="2" t="s">
         <v>239</v>
       </c>
-      <c r="Q126" t="s">
+      <c r="Q126" s="2" t="s">
         <v>240</v>
       </c>
-      <c r="T126" t="s">
+      <c r="T126" s="2" t="s">
         <v>101</v>
       </c>
-      <c r="U126" t="s">
+      <c r="U126" s="2" t="s">
         <v>241</v>
       </c>
     </row>

</xml_diff>